<commit_message>
added mail to approver values for robotest
</commit_message>
<xml_diff>
--- a/newstart/Infra_CMDB_Template.xlsx
+++ b/newstart/Infra_CMDB_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
   <si>
     <t>Server Name</t>
   </si>
@@ -112,37 +112,40 @@
     <t>Lokesh Kumar Kannan</t>
   </si>
   <si>
-    <t>surya</t>
+    <t>suryakumar.r@businesscoresolutions.com</t>
+  </si>
+  <si>
+    <t>madhusoodhanan.p@businesscoresoltuions.com</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>SAP_REPLAY_MAESTRO</t>
+  </si>
+  <si>
+    <t>3.221.134.66</t>
+  </si>
+  <si>
+    <t>Functinonal</t>
+  </si>
+  <si>
+    <t>Windows</t>
+  </si>
+  <si>
+    <t>test</t>
   </si>
   <si>
     <t>Madhusoodhan</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
-  <si>
-    <t>SAP_REPLAY_MAESTRO</t>
-  </si>
-  <si>
-    <t>3.221.134.66</t>
-  </si>
-  <si>
-    <t>Functinonal</t>
-  </si>
-  <si>
-    <t>Windows</t>
-  </si>
-  <si>
-    <t>test</t>
   </si>
   <si>
     <t>Sanbox2</t>
@@ -240,7 +243,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -269,20 +272,11 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -607,31 +601,31 @@
   <dimension ref="A1:V6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="15" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="16" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="15" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="18" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="17" width="21.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="17" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="19" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="17" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="17" width="8.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="17" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="17" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="17" width="6.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="20" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="20" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="17" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="17" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="17" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="13" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="15" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="14" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="14" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="16" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="14" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="14" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="14" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="14" width="6.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="17" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="14" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="14" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="14" width="6.2907142857142855" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -699,7 +693,7 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -767,7 +761,7 @@
         <v>37</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="8" t="s">
         <v>38</v>
       </c>
@@ -812,7 +806,7 @@
         <v>31</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="Q3" s="3" t="s">
         <v>34</v>
@@ -824,23 +818,23 @@
       <c r="V3" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="11">
+      <c r="A4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="2">
         <v>987654321</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>44</v>
+      <c r="C4" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="4">
         <v>987654321</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>40</v>
@@ -848,7 +842,7 @@
       <c r="H4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="13"/>
+      <c r="I4" s="10"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3" t="s">
         <v>28</v>
@@ -857,36 +851,36 @@
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
       <c r="O4" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P4" s="3" t="s">
         <v>31</v>
       </c>
       <c r="Q4" s="3"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="11">
+      <c r="A5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="2">
         <v>123456789</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>48</v>
+      <c r="C5" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="4">
         <v>123456789</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>40</v>
@@ -894,7 +888,7 @@
       <c r="H5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="13"/>
+      <c r="I5" s="10"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
         <v>28</v>
@@ -906,33 +900,33 @@
         <v>31</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="Q5" s="3"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" s="11">
+      <c r="A6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2">
         <v>918237645</v>
       </c>
-      <c r="C6" s="10" t="s">
-        <v>51</v>
+      <c r="C6" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="4">
         <v>918273465</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>40</v>
@@ -940,7 +934,7 @@
       <c r="H6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="13"/>
+      <c r="I6" s="10"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="s">
         <v>28</v>
@@ -949,14 +943,14 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="P6" s="3" t="s">
         <v>31</v>
       </c>
       <c r="Q6" s="3"/>
-      <c r="R6" s="14"/>
-      <c r="S6" s="14"/>
+      <c r="R6" s="11"/>
+      <c r="S6" s="11"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>

</xml_diff>

<commit_message>
changed the code and the value in excel
</commit_message>
<xml_diff>
--- a/newstart/Infra_CMDB_Template.xlsx
+++ b/newstart/Infra_CMDB_Template.xlsx
@@ -112,7 +112,7 @@
     <t>Lokesh Kumar Kannan</t>
   </si>
   <si>
-    <t>suryakumar.r@businesscoresolutions.com</t>
+    <t>murugan.m@businesscoresolutions.com</t>
   </si>
   <si>
     <t>madhusoodhanan.p@businesscoresoltuions.com</t>
@@ -183,7 +183,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -207,12 +207,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="-Apple-System"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -243,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -272,12 +266,6 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -291,10 +279,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -601,28 +589,28 @@
   <dimension ref="A1:V6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="12" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="13" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="15" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="14" width="21.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="14" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="16" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="14" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="14" width="8.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="14" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="14" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="14" width="6.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="17" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="14" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="14" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="14" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="10" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="11" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="14" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="12" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="12" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="12" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="12" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="12" width="6.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="15" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="12" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="12" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="12" width="6.2907142857142855" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -842,7 +830,7 @@
       <c r="H4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="10"/>
+      <c r="I4" s="7"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3" t="s">
         <v>28</v>
@@ -857,8 +845,8 @@
         <v>31</v>
       </c>
       <c r="Q4" s="3"/>
-      <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
       <c r="T4" s="3"/>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
@@ -888,7 +876,7 @@
       <c r="H5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="10"/>
+      <c r="I5" s="7"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
         <v>28</v>
@@ -903,8 +891,8 @@
         <v>43</v>
       </c>
       <c r="Q5" s="3"/>
-      <c r="R5" s="11"/>
-      <c r="S5" s="11"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
       <c r="T5" s="3"/>
       <c r="U5" s="3"/>
       <c r="V5" s="3"/>
@@ -934,7 +922,7 @@
       <c r="H6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="10"/>
+      <c r="I6" s="7"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="s">
         <v>28</v>
@@ -949,8 +937,8 @@
         <v>31</v>
       </c>
       <c r="Q6" s="3"/>
-      <c r="R6" s="11"/>
-      <c r="S6" s="11"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="6"/>
       <c r="T6" s="3"/>
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>

</xml_diff>

<commit_message>
new vm value added
</commit_message>
<xml_diff>
--- a/newstart/Infra_CMDB_Template.xlsx
+++ b/newstart/Infra_CMDB_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="58">
   <si>
     <t>Server Name</t>
   </si>
@@ -82,40 +82,52 @@
     <t>Notes</t>
   </si>
   <si>
+    <t>metsalab</t>
+  </si>
+  <si>
+    <t>i-0579c298976aff928</t>
+  </si>
+  <si>
+    <t>AWS</t>
+  </si>
+  <si>
+    <t>testing vm from madhan</t>
+  </si>
+  <si>
+    <t>MSD</t>
+  </si>
+  <si>
+    <t>Ubuntu</t>
+  </si>
+  <si>
+    <t>us-east-1</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>murugan.m@businesscoresolutions.com</t>
+  </si>
+  <si>
+    <t>madhusoodhanan.p@businesscoresolutions.com</t>
+  </si>
+  <si>
     <t>robotest</t>
   </si>
   <si>
     <t>i-08b529c38bee4ad32</t>
   </si>
   <si>
-    <t>AWS</t>
-  </si>
-  <si>
     <t>Python Team Test Server</t>
   </si>
   <si>
     <t>Sandbox</t>
   </si>
   <si>
-    <t>Ubuntu</t>
-  </si>
-  <si>
-    <t>us-east-1</t>
-  </si>
-  <si>
-    <t>Python</t>
-  </si>
-  <si>
     <t>Symphony FastAPI</t>
   </si>
   <si>
     <t>Lokesh Kumar Kannan</t>
-  </si>
-  <si>
-    <t>murugan.m@businesscoresolutions.com</t>
-  </si>
-  <si>
-    <t>madhusoodhanan.p@businesscoresolutions.com</t>
   </si>
   <si>
     <t>Active</t>
@@ -237,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -255,6 +267,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
@@ -586,31 +613,31 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="10" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="13" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="12" width="21.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="12" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="12" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="14" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="12" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="12" width="8.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="12" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="12" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="12" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="12" width="6.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="15" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="15" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="12" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="12" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="12" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="15" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="16" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="15" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="18" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="17" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="17" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="19" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="17" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="17" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="17" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="17" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="17" width="6.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="20" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="20" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="17" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="17" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="17" width="6.2907142857142855" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -681,21 +708,21 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="16.5">
+      <c r="A2" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="4">
-        <v>637423361475</v>
+      <c r="E2" s="9">
+        <v>71331301700</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>25</v>
@@ -706,58 +733,38 @@
       <c r="H2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="7">
-        <v>2.3</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>24</v>
-      </c>
+      <c r="I2" s="10"/>
+      <c r="J2" s="3"/>
       <c r="K2" s="3" t="s">
         <v>28</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="P2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="R2" s="6">
-        <v>45658</v>
-      </c>
-      <c r="S2" s="6">
-        <v>45876</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>37</v>
-      </c>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>38</v>
+      <c r="A3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>24</v>
@@ -766,15 +773,17 @@
         <v>637423361475</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="I3" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="I3" s="12">
+        <v>2.3</v>
+      </c>
       <c r="J3" s="3" t="s">
         <v>24</v>
       </c>
@@ -782,69 +791,89 @@
         <v>28</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="M3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="P3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="Q3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="R3" s="6"/>
-      <c r="S3" s="6"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
+        <v>38</v>
+      </c>
+      <c r="R3" s="6">
+        <v>45658</v>
+      </c>
+      <c r="S3" s="6">
+        <v>45876</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B4" s="2">
-        <v>987654321</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>45</v>
+      <c r="A4" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>42</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E4" s="4">
-        <v>987654321</v>
+        <v>637423361475</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="7"/>
-      <c r="J4" s="3"/>
+        <v>45</v>
+      </c>
+      <c r="I4" s="12"/>
+      <c r="J4" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="K4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
+      <c r="L4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>37</v>
+      </c>
       <c r="O4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="P4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q4" s="3"/>
+      <c r="Q4" s="3" t="s">
+        <v>38</v>
+      </c>
       <c r="R4" s="6"/>
       <c r="S4" s="6"/>
       <c r="T4" s="3"/>
@@ -856,7 +885,7 @@
         <v>48</v>
       </c>
       <c r="B5" s="2">
-        <v>123456789</v>
+        <v>987654321</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>49</v>
@@ -865,18 +894,18 @@
         <v>24</v>
       </c>
       <c r="E5" s="4">
-        <v>123456789</v>
+        <v>987654321</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>50</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="7"/>
+        <v>45</v>
+      </c>
+      <c r="I5" s="12"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3" t="s">
         <v>28</v>
@@ -885,10 +914,10 @@
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
       <c r="O5" s="3" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="Q5" s="3"/>
       <c r="R5" s="6"/>
@@ -899,30 +928,30 @@
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B6" s="2">
-        <v>918237645</v>
+        <v>123456789</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="4">
-        <v>918273465</v>
+        <v>123456789</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="7"/>
+      <c r="I6" s="12"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="s">
         <v>28</v>
@@ -931,10 +960,10 @@
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
       <c r="O6" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P6" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="Q6" s="3"/>
       <c r="R6" s="6"/>
@@ -943,6 +972,52 @@
       <c r="U6" s="3"/>
       <c r="V6" s="3"/>
     </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+      <c r="A7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="2">
+        <v>918237645</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="4">
+        <v>918273465</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="12"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="6"/>
+      <c r="S7" s="6"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
having issue with intger in account
</commit_message>
<xml_diff>
--- a/newstart/Infra_CMDB_Template.xlsx
+++ b/newstart/Infra_CMDB_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="60">
   <si>
     <t>Server Name</t>
   </si>
@@ -91,6 +91,9 @@
     <t>AWS</t>
   </si>
   <si>
+    <t>071331301700</t>
+  </si>
+  <si>
     <t>testing vm from madhan</t>
   </si>
   <si>
@@ -164,6 +167,9 @@
   </si>
   <si>
     <t>Sandbox2</t>
+  </si>
+  <si>
+    <t>0987654321</t>
   </si>
   <si>
     <t>Sb2</t>
@@ -194,7 +200,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -205,7 +213,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -249,7 +257,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -257,16 +265,37 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -275,41 +304,17 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="14" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -342,7 +347,7 @@
         <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4F818D"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="C0504D"/>
@@ -616,31 +621,31 @@
   <dimension ref="A1:V7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="15" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="16" width="12.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="15" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="17" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="18" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="17" width="21.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="17" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="17" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="19" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="17" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="17" width="8.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="17" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="17" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="17" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="17" width="6.433571428571429" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="20" width="13.290714285714287" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="20" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="17" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="17" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="17" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="14" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="15" width="12.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="14" width="25.290714285714284" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="17" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="16" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="16" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="18" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="16" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="16" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="16" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="16" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="16" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="16" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="16" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="16" width="6.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="19" width="13.290714285714287" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="19" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="16" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="16" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="16" width="6.2907142857142855" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="16.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -650,373 +655,373 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="3" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="16.5">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="9">
-        <v>71331301700</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="G2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="10"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3" t="s">
+      <c r="H2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="I2" s="7"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3" t="s">
+      <c r="L2" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="11"/>
-      <c r="S2" s="11"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
+      <c r="P2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" s="8"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="8"/>
+      <c r="U2" s="8"/>
+      <c r="V2" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="16.5">
       <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" s="3">
+        <v>637423361475</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" s="10">
+        <v>2.3</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="4">
-        <v>637423361475</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="12">
-        <v>2.3</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="R3" s="6">
-        <v>45658</v>
-      </c>
-      <c r="S3" s="6">
-        <v>45876</v>
-      </c>
-      <c r="T3" s="3" t="s">
+      <c r="Q3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="U3" s="3" t="s">
+      <c r="R3" s="11">
+        <v>25569.22969511574</v>
+      </c>
+      <c r="S3" s="11">
+        <v>25569.22969763889</v>
+      </c>
+      <c r="T3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="V3" s="3" t="s">
+      <c r="U3" s="1" t="s">
         <v>41</v>
+      </c>
+      <c r="V3" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="B4" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>637423361475</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="H4" s="3" t="s">
+      <c r="F4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="12"/>
-      <c r="J4" s="3" t="s">
+      <c r="H4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I4" s="7"/>
+      <c r="J4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="N4" s="3" t="s">
+      <c r="K4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="O4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q4" s="3" t="s">
+      <c r="N4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="6"/>
-      <c r="S4" s="6"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
+      <c r="O4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="8"/>
+      <c r="U4" s="8"/>
+      <c r="V4" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="16.5">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B5" s="2">
         <v>987654321</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="4">
-        <v>987654321</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" s="3" t="s">
+      <c r="E5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="I5" s="12"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="6"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
+      <c r="H5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="7"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="8"/>
+      <c r="U5" s="8"/>
+      <c r="V5" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="16.5">
       <c r="A6" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B6" s="2">
         <v>123456789</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6" s="3">
         <v>123456789</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="12"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3" t="s">
+      <c r="F6" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="3"/>
-      <c r="U6" s="3"/>
-      <c r="V6" s="3"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="16.5">
       <c r="A7" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B7" s="2">
         <v>918237645</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7" s="3">
         <v>918273465</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3" t="s">
+      <c r="F7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q7" s="3"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6"/>
-      <c r="T7" s="3"/>
-      <c r="U7" s="3"/>
-      <c r="V7" s="3"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="8"/>
+      <c r="V7" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added 0 to accounts
</commit_message>
<xml_diff>
--- a/newstart/Infra_CMDB_Template.xlsx
+++ b/newstart/Infra_CMDB_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="61">
   <si>
     <t>Server Name</t>
   </si>
@@ -182,6 +182,9 @@
   </si>
   <si>
     <t>sandbox3</t>
+  </si>
+  <si>
+    <t>0123456789</t>
   </si>
   <si>
     <t>Sv2</t>
@@ -304,13 +307,13 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -624,25 +627,25 @@
     <col min="1" max="1" style="14" width="25.290714285714284" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="15" width="12.719285714285713" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="14" width="25.290714285714284" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="16" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="17" width="16.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="16" width="21.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="16" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="16" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="18" width="10.719285714285713" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="16" width="14.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="16" width="8.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="16" width="13.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="16" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="16" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="16" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="16" width="20.14785714285714" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="16" width="6.433571428571429" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="14" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="16" width="16.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="14" width="21.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="14" width="9.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="17" width="10.719285714285713" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="18" width="14.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="14" width="8.862142857142858" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="18" width="13.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="18" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="18" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="14" width="20.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="18" width="6.433571428571429" customWidth="1" bestFit="1"/>
     <col min="18" max="18" style="19" width="13.290714285714287" customWidth="1" bestFit="1"/>
     <col min="19" max="19" style="19" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="16" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="16" width="18.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="16" width="6.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="18" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="18" width="18.719285714285714" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="18" width="6.2907142857142855" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="16.5">
@@ -814,10 +817,10 @@
         <v>39</v>
       </c>
       <c r="R3" s="11">
-        <v>25569.22969511574</v>
+        <v>25569.229462604166</v>
       </c>
       <c r="S3" s="11">
-        <v>25569.22969763889</v>
+        <v>25569.229462604166</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>40</v>
@@ -944,11 +947,11 @@
       <c r="D6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="3">
-        <v>123456789</v>
+      <c r="E6" s="6" t="s">
+        <v>56</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>45</v>
@@ -979,13 +982,13 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="16.5">
       <c r="A7" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2">
         <v>918237645</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>24</v>
@@ -994,7 +997,7 @@
         <v>918273465</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>45</v>

</xml_diff>

<commit_message>
added lokesh anna mail
</commit_message>
<xml_diff>
--- a/newstart/Infra_CMDB_Template.xlsx
+++ b/newstart/Infra_CMDB_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
   <si>
     <t>Server Name</t>
   </si>
@@ -109,28 +109,31 @@
     <t>Python</t>
   </si>
   <si>
+    <t>lokeshkumar.k@businesscoresolutions.com</t>
+  </si>
+  <si>
+    <t>madhusoodhanan.p@businesscoresolutions.com</t>
+  </si>
+  <si>
+    <t>robotest</t>
+  </si>
+  <si>
+    <t>i-08b529c38bee4ad32</t>
+  </si>
+  <si>
+    <t>Python Team Test Server</t>
+  </si>
+  <si>
+    <t>Sandbox</t>
+  </si>
+  <si>
+    <t>Symphony FastAPI</t>
+  </si>
+  <si>
+    <t>Lokesh Kumar Kannan</t>
+  </si>
+  <si>
     <t>murugan.m@businesscoresolutions.com</t>
-  </si>
-  <si>
-    <t>madhusoodhanan.p@businesscoresolutions.com</t>
-  </si>
-  <si>
-    <t>robotest</t>
-  </si>
-  <si>
-    <t>i-08b529c38bee4ad32</t>
-  </si>
-  <si>
-    <t>Python Team Test Server</t>
-  </si>
-  <si>
-    <t>Sandbox</t>
-  </si>
-  <si>
-    <t>Symphony FastAPI</t>
-  </si>
-  <si>
-    <t>Lokesh Kumar Kannan</t>
   </si>
   <si>
     <t>Active</t>
@@ -206,13 +209,19 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -280,14 +289,14 @@
     <xf xfId="0" numFmtId="49" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -295,10 +304,10 @@
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -648,7 +657,7 @@
     <col min="22" max="22" style="18" width="6.2907142857142855" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -716,7 +725,7 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -764,7 +773,7 @@
       <c r="U2" s="8"/>
       <c r="V2" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="1" t="s">
         <v>33</v>
       </c>
@@ -808,39 +817,39 @@
         <v>38</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="P3" s="1" t="s">
         <v>32</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R3" s="11">
-        <v>25569.229462604166</v>
+        <v>25569.22946759259</v>
       </c>
       <c r="S3" s="11">
-        <v>25569.229462604166</v>
+        <v>25569.22946759259</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>44</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>43</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>24</v>
@@ -849,13 +858,13 @@
         <v>637423361475</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I4" s="7"/>
       <c r="J4" s="1" t="s">
@@ -865,7 +874,7 @@
         <v>29</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>37</v>
@@ -877,10 +886,10 @@
         <v>38</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="R4" s="9"/>
       <c r="S4" s="9"/>
@@ -888,30 +897,30 @@
       <c r="U4" s="8"/>
       <c r="V4" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B5" s="2">
         <v>987654321</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>24</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I5" s="7"/>
       <c r="J5" s="8"/>
@@ -922,7 +931,7 @@
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
       <c r="O5" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P5" s="1" t="s">
         <v>38</v>
@@ -934,27 +943,27 @@
       <c r="U5" s="8"/>
       <c r="V5" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2">
         <v>123456789</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>28</v>
@@ -971,7 +980,7 @@
         <v>38</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Q6" s="8"/>
       <c r="R6" s="9"/>
@@ -980,15 +989,15 @@
       <c r="U6" s="8"/>
       <c r="V6" s="8"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="16.5">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2">
         <v>918237645</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>24</v>
@@ -997,10 +1006,10 @@
         <v>918273465</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>28</v>
@@ -1014,7 +1023,7 @@
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="P7" s="1" t="s">
         <v>38</v>

</xml_diff>